<commit_message>
Auto update ETF comparison: Mon Apr 27 08:17:50 UTC 2026
</commit_message>
<xml_diff>
--- a/data/00981A/20260427.xlsx
+++ b/data/00981A/20260427.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="234">
-  <si>
-    <t xml:space="preserve">資料日期：115/04/24</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="228">
+  <si>
+    <t xml:space="preserve">資料日期：115/04/27</t>
   </si>
   <si>
     <t xml:space="preserve">基金資產</t>
@@ -23,19 +23,19 @@
     <t xml:space="preserve">淨資產</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 212,076,376,428</t>
+    <t xml:space="preserve">NTD 232,148,514,804</t>
   </si>
   <si>
     <t xml:space="preserve">流通在外單位數</t>
   </si>
   <si>
-    <t xml:space="preserve">7,672,209,000</t>
+    <t xml:space="preserve">8,369,209,000</t>
   </si>
   <si>
     <t xml:space="preserve">每單位淨值</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 27.64</t>
+    <t xml:space="preserve">NTD 27.74</t>
   </si>
   <si>
     <t xml:space="preserve">項目</t>
@@ -59,19 +59,19 @@
     <t xml:space="preserve">股票</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 200,526,562,520</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.55%</t>
+    <t xml:space="preserve">NTD 214,951,390,490</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.59%</t>
   </si>
   <si>
     <t xml:space="preserve">現金</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 14,740,905,754</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.95%</t>
+    <t xml:space="preserve">NTD 15,329,426,136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.60%</t>
   </si>
   <si>
     <t xml:space="preserve">期貨保證金</t>
@@ -80,7 +80,7 @@
     <t xml:space="preserve">NTD 500,128,241</t>
   </si>
   <si>
-    <t xml:space="preserve">0.24%</t>
+    <t xml:space="preserve">0.22%</t>
   </si>
   <si>
     <t xml:space="preserve">申贖應付款</t>
@@ -89,10 +89,10 @@
     <t xml:space="preserve">應收付證券款</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD -11,033,251,389</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.20%</t>
+    <t xml:space="preserve">NTD -21,933,220,529</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-9.45%</t>
   </si>
   <si>
     <t xml:space="preserve">股票代號</t>
@@ -113,10 +113,10 @@
     <t xml:space="preserve">台積電</t>
   </si>
   <si>
-    <t xml:space="preserve">9,114,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.39%</t>
+    <t xml:space="preserve">9,693,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.46%</t>
   </si>
   <si>
     <t xml:space="preserve">2383</t>
@@ -125,10 +125,22 @@
     <t xml:space="preserve">台光電</t>
   </si>
   <si>
-    <t xml:space="preserve">4,125,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.70%</t>
+    <t xml:space="preserve">4,425,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.02%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">智邦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,031,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.65%</t>
   </si>
   <si>
     <t xml:space="preserve">2308</t>
@@ -140,7 +152,43 @@
     <t xml:space="preserve">6,024,000</t>
   </si>
   <si>
-    <t xml:space="preserve">5.89%</t>
+    <t xml:space="preserve">5.24%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金像電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8,240,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.04%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">南電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12,637,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.97%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3665</t>
+  </si>
+  <si>
+    <t xml:space="preserve">貿聯-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,377,848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.96%</t>
   </si>
   <si>
     <t xml:space="preserve">3653</t>
@@ -152,7 +200,7 @@
     <t xml:space="preserve">2,267,000</t>
   </si>
   <si>
-    <t xml:space="preserve">5.74%</t>
+    <t xml:space="preserve">4.84%</t>
   </si>
   <si>
     <t xml:space="preserve">3017</t>
@@ -164,55 +212,7 @@
     <t xml:space="preserve">3,902,000</t>
   </si>
   <si>
-    <t xml:space="preserve">5.42%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3665</t>
-  </si>
-  <si>
-    <t xml:space="preserve">貿聯-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,097,848</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.34%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">智邦</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,231,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.28%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2368</t>
-  </si>
-  <si>
-    <t xml:space="preserve">金像電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,748,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.08%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">南電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11,881,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.90%</t>
+    <t xml:space="preserve">4.77%</t>
   </si>
   <si>
     <t xml:space="preserve">2454</t>
@@ -221,10 +221,10 @@
     <t xml:space="preserve">聯發科</t>
   </si>
   <si>
-    <t xml:space="preserve">3,867,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.44%</t>
+    <t xml:space="preserve">4,147,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.35%</t>
   </si>
   <si>
     <t xml:space="preserve">6223</t>
@@ -233,10 +233,10 @@
     <t xml:space="preserve">旺矽</t>
   </si>
   <si>
-    <t xml:space="preserve">1,774,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.89%</t>
+    <t xml:space="preserve">1,886,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.96%</t>
   </si>
   <si>
     <t xml:space="preserve">3037</t>
@@ -248,7 +248,19 @@
     <t xml:space="preserve">9,287,000</t>
   </si>
   <si>
-    <t xml:space="preserve">3.46%</t>
+    <t xml:space="preserve">3.36%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6669</t>
+  </si>
+  <si>
+    <t xml:space="preserve">緯穎</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,549,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.26%</t>
   </si>
   <si>
     <t xml:space="preserve">5274</t>
@@ -257,22 +269,10 @@
     <t xml:space="preserve">信驊</t>
   </si>
   <si>
-    <t xml:space="preserve">351,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.71%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6669</t>
-  </si>
-  <si>
-    <t xml:space="preserve">緯穎</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,101,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.41%</t>
+    <t xml:space="preserve">373,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.57%</t>
   </si>
   <si>
     <t xml:space="preserve">2327</t>
@@ -281,22 +281,34 @@
     <t xml:space="preserve">國巨*</t>
   </si>
   <si>
-    <t xml:space="preserve">14,288,000</t>
+    <t xml:space="preserve">15,196,000</t>
   </si>
   <si>
     <t xml:space="preserve">2.00%</t>
   </si>
   <si>
+    <t xml:space="preserve">6805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">富世達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,099,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.87%</t>
+  </si>
+  <si>
     <t xml:space="preserve">3711</t>
   </si>
   <si>
     <t xml:space="preserve">日月光投控</t>
   </si>
   <si>
-    <t xml:space="preserve">7,654,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.79%</t>
+    <t xml:space="preserve">8,174,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.74%</t>
   </si>
   <si>
     <t xml:space="preserve">6515</t>
@@ -305,22 +317,10 @@
     <t xml:space="preserve">穎崴</t>
   </si>
   <si>
-    <t xml:space="preserve">368,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.75%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">富世達</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,698,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.53%</t>
+    <t xml:space="preserve">391,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.61%</t>
   </si>
   <si>
     <t xml:space="preserve">6510</t>
@@ -329,10 +329,34 @@
     <t xml:space="preserve">精測</t>
   </si>
   <si>
-    <t xml:space="preserve">875,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.50%</t>
+    <t xml:space="preserve">930,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.43%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">京元電子</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11,172,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.36%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3661</t>
+  </si>
+  <si>
+    <t xml:space="preserve">世芯-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">738,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.32%</t>
   </si>
   <si>
     <t xml:space="preserve">6274</t>
@@ -344,31 +368,7 @@
     <t xml:space="preserve">3,019,000</t>
   </si>
   <si>
-    <t xml:space="preserve">1.49%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">京元電子</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,503,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.42%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3661</t>
-  </si>
-  <si>
-    <t xml:space="preserve">世芯-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">694,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.38%</t>
+    <t xml:space="preserve">1.29%</t>
   </si>
   <si>
     <t xml:space="preserve">3189</t>
@@ -377,10 +377,22 @@
     <t xml:space="preserve">景碩</t>
   </si>
   <si>
-    <t xml:space="preserve">5,038,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.25%</t>
+    <t xml:space="preserve">5,358,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.19%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">鴻海</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,727,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.05%</t>
   </si>
   <si>
     <t xml:space="preserve">2303</t>
@@ -389,10 +401,10 @@
     <t xml:space="preserve">聯電</t>
   </si>
   <si>
-    <t xml:space="preserve">30,837,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.08%</t>
+    <t xml:space="preserve">32,791,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.03%</t>
   </si>
   <si>
     <t xml:space="preserve">8358</t>
@@ -404,19 +416,7 @@
     <t xml:space="preserve">5,558,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.94%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">鴻海</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,927,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.72%</t>
+    <t xml:space="preserve">0.80%</t>
   </si>
   <si>
     <t xml:space="preserve">8210</t>
@@ -425,10 +425,43 @@
     <t xml:space="preserve">勤誠</t>
   </si>
   <si>
-    <t xml:space="preserve">1,051,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.60%</t>
+    <t xml:space="preserve">1,117,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.56%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">高技</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,130,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.50%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">創意</t>
+  </si>
+  <si>
+    <t xml:space="preserve">271,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.46%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">漢唐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,091,000</t>
   </si>
   <si>
     <t xml:space="preserve">6147</t>
@@ -440,43 +473,7 @@
     <t xml:space="preserve">7,884,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.54%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3443</t>
-  </si>
-  <si>
-    <t xml:space="preserve">創意</t>
-  </si>
-  <si>
-    <t xml:space="preserve">271,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.52%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">漢唐</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,091,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.51%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">高技</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,880,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.50%</t>
+    <t xml:space="preserve">0.44%</t>
   </si>
   <si>
     <t xml:space="preserve">3264</t>
@@ -485,10 +482,10 @@
     <t xml:space="preserve">欣銓</t>
   </si>
   <si>
-    <t xml:space="preserve">4,896,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.48%</t>
+    <t xml:space="preserve">4,897,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.41%</t>
   </si>
   <si>
     <t xml:space="preserve">8996</t>
@@ -500,7 +497,7 @@
     <t xml:space="preserve">535,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.28%</t>
+    <t xml:space="preserve">0.25%</t>
   </si>
   <si>
     <t xml:space="preserve">7769</t>
@@ -509,10 +506,10 @@
     <t xml:space="preserve">鴻勁</t>
   </si>
   <si>
-    <t xml:space="preserve">97,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.22%</t>
+    <t xml:space="preserve">98,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.21%</t>
   </si>
   <si>
     <t xml:space="preserve">6191</t>
@@ -521,10 +518,10 @@
     <t xml:space="preserve">精成科</t>
   </si>
   <si>
-    <t xml:space="preserve">3,985,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.20%</t>
+    <t xml:space="preserve">3,986,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18%</t>
   </si>
   <si>
     <t xml:space="preserve">2481</t>
@@ -533,10 +530,67 @@
     <t xml:space="preserve">強茂</t>
   </si>
   <si>
-    <t xml:space="preserve">3,651,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.17%</t>
+    <t xml:space="preserve">3,652,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.16%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3376</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新日興</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,681,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6415</t>
+  </si>
+  <si>
+    <t xml:space="preserve">矽力*-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">660,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4966</t>
+  </si>
+  <si>
+    <t xml:space="preserve">譜瑞-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">371,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6488</t>
+  </si>
+  <si>
+    <t xml:space="preserve">環球晶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">333,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.09%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">華通</t>
+  </si>
+  <si>
+    <t xml:space="preserve">843,000</t>
   </si>
   <si>
     <t xml:space="preserve">3211</t>
@@ -545,76 +599,7 @@
     <t xml:space="preserve">順達</t>
   </si>
   <si>
-    <t xml:space="preserve">916,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.16%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3376</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新日興</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,561,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6415</t>
-  </si>
-  <si>
-    <t xml:space="preserve">矽力*-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">660,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.14%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4966</t>
-  </si>
-  <si>
-    <t xml:space="preserve">譜瑞-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">370,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.11%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3324</t>
-  </si>
-  <si>
-    <t xml:space="preserve">雙鴻</t>
-  </si>
-  <si>
-    <t xml:space="preserve">170,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.10%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6488</t>
-  </si>
-  <si>
-    <t xml:space="preserve">環球晶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">332,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.09%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2313</t>
-  </si>
-  <si>
-    <t xml:space="preserve">華通</t>
-  </si>
-  <si>
-    <t xml:space="preserve">764,000</t>
+    <t xml:space="preserve">458,000</t>
   </si>
   <si>
     <t xml:space="preserve">0.08%</t>
@@ -626,10 +611,10 @@
     <t xml:space="preserve">優群</t>
   </si>
   <si>
-    <t xml:space="preserve">780,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.07%</t>
+    <t xml:space="preserve">830,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.06%</t>
   </si>
   <si>
     <t xml:space="preserve">1303</t>
@@ -638,10 +623,10 @@
     <t xml:space="preserve">南亞</t>
   </si>
   <si>
-    <t xml:space="preserve">1,373,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.06%</t>
+    <t xml:space="preserve">1,374,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.05%</t>
   </si>
   <si>
     <t xml:space="preserve">2002</t>
@@ -650,10 +635,10 @@
     <t xml:space="preserve">中鋼</t>
   </si>
   <si>
-    <t xml:space="preserve">5,160,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.05%</t>
+    <t xml:space="preserve">5,161,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.04%</t>
   </si>
   <si>
     <t xml:space="preserve">1319</t>
@@ -662,12 +647,24 @@
     <t xml:space="preserve">東陽</t>
   </si>
   <si>
-    <t xml:space="preserve">508,000</t>
+    <t xml:space="preserve">509,000</t>
   </si>
   <si>
     <t xml:space="preserve">0.02%</t>
   </si>
   <si>
+    <t xml:space="preserve">2357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">華碩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00%</t>
+  </si>
+  <si>
     <t xml:space="preserve">1815</t>
   </si>
   <si>
@@ -677,21 +674,6 @@
     <t xml:space="preserve">107,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.01%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2357</t>
-  </si>
-  <si>
-    <t xml:space="preserve">華碩</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.00%</t>
-  </si>
-  <si>
     <t xml:space="preserve">2439</t>
   </si>
   <si>
@@ -713,7 +695,7 @@
     <t xml:space="preserve">世界</t>
   </si>
   <si>
-    <t xml:space="preserve">61,000</t>
+    <t xml:space="preserve">62,000</t>
   </si>
 </sst>
 </file>
@@ -792,7 +774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
@@ -874,18 +856,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1514,7 +1484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.9" bestFit="1" customWidth="1" collapsed="1"/>
@@ -2089,119 +2059,119 @@
         <v>149</v>
       </c>
       <c r="D50" s="150" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="151" t="s">
+        <v>150</v>
+      </c>
+      <c r="B51" s="152" t="s">
         <v>151</v>
       </c>
-      <c r="B51" s="152" t="s">
+      <c r="C51" s="153" t="s">
         <v>152</v>
       </c>
-      <c r="C51" s="153" t="s">
+      <c r="D51" s="154" t="s">
         <v>153</v>
-      </c>
-      <c r="D51" s="154" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="155" t="s">
+        <v>154</v>
+      </c>
+      <c r="B52" s="156" t="s">
         <v>155</v>
       </c>
-      <c r="B52" s="156" t="s">
+      <c r="C52" s="157" t="s">
         <v>156</v>
       </c>
-      <c r="C52" s="157" t="s">
+      <c r="D52" s="158" t="s">
         <v>157</v>
-      </c>
-      <c r="D52" s="158" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="159" t="s">
+        <v>158</v>
+      </c>
+      <c r="B53" s="160" t="s">
         <v>159</v>
       </c>
-      <c r="B53" s="160" t="s">
+      <c r="C53" s="161" t="s">
         <v>160</v>
       </c>
-      <c r="C53" s="161" t="s">
+      <c r="D53" s="162" t="s">
         <v>161</v>
-      </c>
-      <c r="D53" s="162" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="163" t="s">
+        <v>162</v>
+      </c>
+      <c r="B54" s="164" t="s">
         <v>163</v>
       </c>
-      <c r="B54" s="164" t="s">
+      <c r="C54" s="165" t="s">
         <v>164</v>
       </c>
-      <c r="C54" s="165" t="s">
+      <c r="D54" s="166" t="s">
         <v>165</v>
-      </c>
-      <c r="D54" s="166" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="167" t="s">
+        <v>166</v>
+      </c>
+      <c r="B55" s="168" t="s">
         <v>167</v>
       </c>
-      <c r="B55" s="168" t="s">
+      <c r="C55" s="169" t="s">
         <v>168</v>
       </c>
-      <c r="C55" s="169" t="s">
+      <c r="D55" s="170" t="s">
         <v>169</v>
-      </c>
-      <c r="D55" s="170" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="171" t="s">
+        <v>170</v>
+      </c>
+      <c r="B56" s="172" t="s">
         <v>171</v>
       </c>
-      <c r="B56" s="172" t="s">
+      <c r="C56" s="173" t="s">
         <v>172</v>
       </c>
-      <c r="C56" s="173" t="s">
+      <c r="D56" s="174" t="s">
         <v>173</v>
-      </c>
-      <c r="D56" s="174" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="175" t="s">
+        <v>174</v>
+      </c>
+      <c r="B57" s="176" t="s">
         <v>175</v>
       </c>
-      <c r="B57" s="176" t="s">
+      <c r="C57" s="177" t="s">
         <v>176</v>
       </c>
-      <c r="C57" s="177" t="s">
+      <c r="D57" s="178" t="s">
         <v>177</v>
-      </c>
-      <c r="D57" s="178" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="179" t="s">
+        <v>178</v>
+      </c>
+      <c r="B58" s="180" t="s">
         <v>179</v>
       </c>
-      <c r="B58" s="180" t="s">
+      <c r="C58" s="181" t="s">
         <v>180</v>
       </c>
-      <c r="C58" s="181" t="s">
+      <c r="D58" s="182" t="s">
         <v>181</v>
-      </c>
-      <c r="D58" s="182" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="59">
@@ -2243,161 +2213,147 @@
         <v>192</v>
       </c>
       <c r="D61" s="194" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="195" t="s">
+        <v>193</v>
+      </c>
+      <c r="B62" s="196" t="s">
         <v>194</v>
       </c>
-      <c r="B62" s="196" t="s">
+      <c r="C62" s="197" t="s">
         <v>195</v>
       </c>
-      <c r="C62" s="197" t="s">
+      <c r="D62" s="198" t="s">
         <v>196</v>
-      </c>
-      <c r="D62" s="198" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="199" t="s">
+        <v>197</v>
+      </c>
+      <c r="B63" s="200" t="s">
         <v>198</v>
       </c>
-      <c r="B63" s="200" t="s">
+      <c r="C63" s="201" t="s">
         <v>199</v>
       </c>
-      <c r="C63" s="201" t="s">
+      <c r="D63" s="202" t="s">
         <v>200</v>
-      </c>
-      <c r="D63" s="202" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="203" t="s">
+        <v>201</v>
+      </c>
+      <c r="B64" s="204" t="s">
         <v>202</v>
       </c>
-      <c r="B64" s="204" t="s">
+      <c r="C64" s="205" t="s">
         <v>203</v>
       </c>
-      <c r="C64" s="205" t="s">
+      <c r="D64" s="206" t="s">
         <v>204</v>
-      </c>
-      <c r="D64" s="206" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="207" t="s">
+        <v>205</v>
+      </c>
+      <c r="B65" s="208" t="s">
         <v>206</v>
       </c>
-      <c r="B65" s="208" t="s">
+      <c r="C65" s="209" t="s">
         <v>207</v>
       </c>
-      <c r="C65" s="209" t="s">
+      <c r="D65" s="210" t="s">
         <v>208</v>
-      </c>
-      <c r="D65" s="210" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="211" t="s">
+        <v>209</v>
+      </c>
+      <c r="B66" s="212" t="s">
         <v>210</v>
       </c>
-      <c r="B66" s="212" t="s">
+      <c r="C66" s="213" t="s">
         <v>211</v>
       </c>
-      <c r="C66" s="213" t="s">
+      <c r="D66" s="214" t="s">
         <v>212</v>
-      </c>
-      <c r="D66" s="214" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="215" t="s">
+        <v>213</v>
+      </c>
+      <c r="B67" s="216" t="s">
         <v>214</v>
       </c>
-      <c r="B67" s="216" t="s">
+      <c r="C67" s="217" t="s">
         <v>215</v>
       </c>
-      <c r="C67" s="217" t="s">
+      <c r="D67" s="218" t="s">
         <v>216</v>
-      </c>
-      <c r="D67" s="218" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="219" t="s">
+        <v>217</v>
+      </c>
+      <c r="B68" s="220" t="s">
         <v>218</v>
       </c>
-      <c r="B68" s="220" t="s">
+      <c r="C68" s="221" t="s">
         <v>219</v>
       </c>
-      <c r="C68" s="221" t="s">
-        <v>220</v>
-      </c>
       <c r="D68" s="222" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="223" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B69" s="224" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C69" s="225" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="D69" s="226" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="227" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B70" s="228" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C70" s="229" t="s">
         <v>224</v>
       </c>
       <c r="D70" s="230" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="231" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B71" s="232" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C71" s="233" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D71" s="234" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="235" t="s">
-        <v>231</v>
-      </c>
-      <c r="B72" s="236" t="s">
-        <v>232</v>
-      </c>
-      <c r="C72" s="237" t="s">
-        <v>233</v>
-      </c>
-      <c r="D72" s="238" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>